<commit_message>
Fix an error in indices of default rows_to_dilute list in the dilute_new_vial() method
Before this fix, the default rows_to_dilute parameter has been equal to (9, 27, 45) and this caused the dilute_new_vial to try to pipette into the vial number 45+9+9=63, which does not exist in a 54-vial plate.
</commit_message>
<xml_diff>
--- a/zeus-pipetter/multicomponent_reaction/0324_mixing_validation/03_27_reapeat_27reactions_outVRF038202303201421.xlsx
+++ b/zeus-pipetter/multicomponent_reaction/0324_mixing_validation/03_27_reapeat_27reactions_outVRF038202303201421.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reactions_0320" sheetId="1" state="visible" r:id="rId1"/>
@@ -1780,7 +1780,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>1848</v>
+        <v>1809</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -1788,7 +1788,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>16699.9</v>
+        <v>18691.6</v>
       </c>
     </row>
     <row r="3">
@@ -1819,7 +1819,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>1981</v>
+        <v>2003</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>9907.6</v>
+        <v>8784</v>
       </c>
     </row>
     <row r="4">
@@ -1858,7 +1858,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>2087</v>
+        <v>2009</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>4494.2</v>
+        <v>8477.6</v>
       </c>
     </row>
     <row r="5">
@@ -1897,7 +1897,7 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>2082</v>
+        <v>1999</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>4749.5</v>
+        <v>8988.299999999999</v>
       </c>
     </row>
     <row r="6">
@@ -1936,7 +1936,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>2082</v>
+        <v>2009</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -1944,7 +1944,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>4749.5</v>
+        <v>8477.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>